<commit_message>
feat: sync all 11 catalog products to backend excel database
</commit_message>
<xml_diff>
--- a/backend/products.xlsx
+++ b/backend/products.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,6 +639,293 @@
         <v>4.9</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>m1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Double Chocolate Muffin</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>double-chocolate-muffin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rich chocolate muffins loaded with premium dark chocolate chips and a soft, moist center.</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>149</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>muffins</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1555507036-ab1f4038808a?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Blueberry Streusel Muffin</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>blueberry-streusel-muffin</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bursting with fresh blueberries and topped with a crunchy, sweet cinnamon streusel crumble.</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>159</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>muffins</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607958996333-41aef7caefaa?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Chocolate Truffle Pastry Slice</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>chocolate-truffle-pastry</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>A decadent slice of dark chocolate truffle cake layered with velvety cocoa ganache.</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>120</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>pastries</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1587314168485-3236d6710814?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cp1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Red Velvet Cupcake</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>red-velvet-cupcake</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fluffy red velvet cupcake base topped with a smooth, swirl of cream cheese frosting.</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>99</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>cupcakes</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1576618148400-f54bed99fcfd?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>b1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fudgy Walnut Brownie</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fudgy-walnut-brownie</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Decadent chocolate brownie with a cracked top crust, rich fudgy center, and crunch walnuts.</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>129</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>brownies</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1564355808539-22fda35bed7e?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fp1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Classic Apple Pie</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>classic-apple-pie</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Flaky pastry crust stuffed with warm spiced apples, cinnamon, and caramel glaze.</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>699</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>fruit-pies</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1519869325930-281384150729?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ck1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chocochip Cookies Pack</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>chocochip-cookies-pack</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Crispy edges with soft centers, loaded heavily with semi-sweet chocolate chunks.</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>199</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>cookies</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1499636136210-6f4ee915583e?auto=format&amp;fit=crop&amp;w=600&amp;q=80</t>
+        </is>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>